<commit_message>
feat: add verified financial calculator module and corrected
</commit_message>
<xml_diff>
--- a/public/phare_template.xlsx
+++ b/public/phare_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\source\repos\phare\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE24B56-8D1C-4B70-BBF1-208DBAF37FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEA52A9-9804-4863-8D34-24550D53F134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Household" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Annual Expenses" sheetId="5" r:id="rId5"/>
     <sheet name="Goals" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -61,9 +61,6 @@
     <t>Family name / Nom de famille</t>
   </si>
   <si>
-    <t>Tremblay</t>
-  </si>
-  <si>
     <t>Province</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
     <t>Combined annual income / Revenu annuel combiné</t>
   </si>
   <si>
-    <t>120000</t>
-  </si>
-  <si>
     <t>Before tax / Avant impôt</t>
   </si>
   <si>
@@ -118,13 +112,16 @@
     <t>Yes / Oui</t>
   </si>
   <si>
+    <t>350 month plus pension from employer</t>
+  </si>
+  <si>
     <t>Do you contribute to RESP? / Contribuez-vous au REEE?</t>
   </si>
   <si>
     <t>No / Non</t>
   </si>
   <si>
-    <t>$500/yr CESG per child</t>
+    <t xml:space="preserve">$500/yr CESG </t>
   </si>
   <si>
     <t>Do you have a TFSA? / Avez-vous un CELI?</t>
@@ -142,54 +139,54 @@
     <t>Ontario</t>
   </si>
   <si>
-    <t>Quebec + Ontario = tax gap</t>
+    <t>Quebec + Ontario = tax gap, Lineu</t>
   </si>
   <si>
     <t>MONTHLY INCOME / REVENU MENSUEL</t>
   </si>
   <si>
+    <t>Enter your MONTHLY take-home pay. Paid bi-weekly? Multiply your paycheque by 2.17. Paid weekly? × 4.33.</t>
+  </si>
+  <si>
+    <t>Entrez votre paie nette MENSUELLE. Payé aux 2 semaines? Multipliez par 2,17. Par semaine? × 4,33.</t>
+  </si>
+  <si>
     <t>Source</t>
   </si>
   <si>
     <t>Member / Membre</t>
   </si>
   <si>
+    <t>Monthly amount / Montant mensuel</t>
+  </si>
+  <si>
+    <t>Salary / Salaire</t>
+  </si>
+  <si>
+    <t>Net monthly (bi-weekly × 2.17)</t>
+  </si>
+  <si>
+    <t>Child benefit / Allocation</t>
+  </si>
+  <si>
+    <t>Household</t>
+  </si>
+  <si>
+    <t>CCB monthly</t>
+  </si>
+  <si>
+    <t>FIXED MONTHLY EXPENSES / DÉPENSES FIXES MENSUELLES</t>
+  </si>
+  <si>
+    <t>Expense / Dépense</t>
+  </si>
+  <si>
+    <t>Category / Catégorie</t>
+  </si>
+  <si>
     <t>Amount / Montant</t>
   </si>
   <si>
-    <t>Frequency / Fréquence</t>
-  </si>
-  <si>
-    <t>Salary / Salaire</t>
-  </si>
-  <si>
-    <t>Bi-weekly / Aux 2 semaines</t>
-  </si>
-  <si>
-    <t>Net pay</t>
-  </si>
-  <si>
-    <t>Child benefit / Allocation enfants</t>
-  </si>
-  <si>
-    <t>Household</t>
-  </si>
-  <si>
-    <t>Monthly / Mensuel</t>
-  </si>
-  <si>
-    <t>CCB</t>
-  </si>
-  <si>
-    <t>FIXED MONTHLY EXPENSES / DÉPENSES FIXES MENSUELLES</t>
-  </si>
-  <si>
-    <t>Expense / Dépense</t>
-  </si>
-  <si>
-    <t>Category / Catégorie</t>
-  </si>
-  <si>
     <t>Account / Compte</t>
   </si>
   <si>
@@ -421,10 +418,13 @@
     <t>December 2026</t>
   </si>
   <si>
+    <t>Doe</t>
+  </si>
+  <si>
     <t>Jeane</t>
   </si>
   <si>
-    <t>Jeanne</t>
+    <t>john</t>
   </si>
   <si>
     <t>John</t>
@@ -440,7 +440,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -471,6 +471,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF6B7280"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="1"/>
     </font>
@@ -529,7 +536,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -538,10 +545,14 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,7 +817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -815,7 +826,7 @@
     <col min="4" max="4" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -843,83 +854,83 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5">
+        <v>2</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5">
+        <v>210</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D11" s="5"/>
     </row>
@@ -931,56 +942,70 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>33</v>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -994,130 +1019,100 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B6" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="6">
-        <v>2500</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="C6" s="7">
+        <v>5958</v>
+      </c>
+      <c r="D6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="4" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="7">
+        <v>5958</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="7">
-        <v>2500</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="B8" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C8" s="7">
+        <v>203.5</v>
+      </c>
+      <c r="D8" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="6">
-        <v>203.5</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1134,9 +1129,9 @@
     <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1145,16 +1140,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -1162,91 +1157,91 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="8">
+        <v>1283.97</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="C4" s="6">
-        <v>1283.97</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="7">
+      <c r="C5" s="9">
         <v>418.94</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="6">
+        <v>53</v>
+      </c>
+      <c r="C6" s="8">
         <v>173.61</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="7">
+        <v>53</v>
+      </c>
+      <c r="C7" s="9">
         <v>318.83</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="8">
+        <v>115.07</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="C8" s="6">
-        <v>115.07</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="7">
+      <c r="C9" s="9">
         <v>176.85</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E9" s="5"/>
     </row>
@@ -1255,13 +1250,13 @@
         <v>129</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="8">
+        <v>134.51</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="C10" s="6">
-        <v>134.51</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="E10" s="4"/>
     </row>
@@ -1270,106 +1265,106 @@
         <v>130</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="9">
+        <v>120.1</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="C11" s="7">
-        <v>120.1</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="6">
+      <c r="C12" s="8">
         <v>182</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" s="7">
+        <v>61</v>
+      </c>
+      <c r="C13" s="9">
         <v>98.55</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="6">
+        <v>53</v>
+      </c>
+      <c r="C14" s="8">
         <v>220.5</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="7">
+      <c r="C15" s="9">
         <v>24.13</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C16" s="6">
+        <v>65</v>
+      </c>
+      <c r="C16" s="8">
         <v>11.49</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="9">
+        <v>78.28</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C17" s="7">
-        <v>78.28</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1421,9 +1416,9 @@
     <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1432,7 +1427,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1441,16 +1436,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>74</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>4</v>
@@ -1458,157 +1453,157 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="9">
+        <v>800</v>
+      </c>
+      <c r="C5" s="9">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="7">
-        <v>800</v>
-      </c>
-      <c r="C5" s="7">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="6">
+        <v>77</v>
+      </c>
+      <c r="B6" s="8">
         <v>500</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="8">
         <v>0</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="7">
+        <v>78</v>
+      </c>
+      <c r="B7" s="9">
         <v>200</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="9">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="8">
+        <v>150</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="B8" s="6">
-        <v>150</v>
-      </c>
-      <c r="C8" s="6">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="7">
+        <v>81</v>
+      </c>
+      <c r="B9" s="9">
         <v>200</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="9">
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B10" s="6">
+        <v>82</v>
+      </c>
+      <c r="B10" s="8">
         <v>100</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="8">
         <v>0</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="7">
+        <v>83</v>
+      </c>
+      <c r="B11" s="9">
         <v>100</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="9">
         <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="6">
+        <v>83</v>
+      </c>
+      <c r="B12" s="8">
         <v>100</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="8">
         <v>0</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="9">
+        <v>150</v>
+      </c>
+      <c r="C13" s="9">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="B13" s="7">
-        <v>150</v>
-      </c>
-      <c r="C13" s="7">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="6">
+        <v>86</v>
+      </c>
+      <c r="B14" s="8">
         <v>100</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="8">
         <v>0</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E14" s="4"/>
     </row>
@@ -1649,9 +1644,9 @@
     <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1661,7 +1656,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1671,7 +1666,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1681,19 +1676,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>4</v>
@@ -1701,142 +1696,142 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="6">
+        <v>93</v>
+      </c>
+      <c r="B6" s="8">
         <v>4200</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="8">
         <f t="shared" ref="C6:C12" si="0">B6/12</f>
         <v>350</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" s="7">
+        <v>96</v>
+      </c>
+      <c r="B7" s="9">
         <v>350</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="9">
         <f t="shared" si="0"/>
         <v>29.166666666666668</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B8" s="6">
+        <v>98</v>
+      </c>
+      <c r="B8" s="8">
         <v>2000</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="8">
         <f t="shared" si="0"/>
         <v>166.66666666666666</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="7">
+        <v>101</v>
+      </c>
+      <c r="B9" s="9">
         <v>800</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="9">
         <f t="shared" si="0"/>
         <v>66.666666666666671</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="6">
+        <v>104</v>
+      </c>
+      <c r="B10" s="8">
         <v>1000</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="8">
         <f t="shared" si="0"/>
         <v>83.333333333333329</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="7">
+        <v>106</v>
+      </c>
+      <c r="B11" s="9">
         <v>1500</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="9">
         <f t="shared" si="0"/>
         <v>125</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B12" s="6">
+        <v>109</v>
+      </c>
+      <c r="B12" s="8">
         <v>1000</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="8">
         <f t="shared" si="0"/>
         <v>83.333333333333329</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F12" s="4"/>
     </row>
@@ -1857,14 +1852,14 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B15" s="9">
+      <c r="A15" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="11">
         <f>SUM(B6:B14)</f>
         <v>10850</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="11">
         <f>SUM(C6:C14)</f>
         <v>904.16666666666674</v>
       </c>
@@ -1889,9 +1884,9 @@
     <col min="2" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1900,30 +1895,30 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" s="8">
+        <v>5200</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="B4" s="6">
-        <v>5200</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -1932,28 +1927,28 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" s="9">
+        <v>8000</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B5" s="7">
-        <v>8000</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>1500</v>
       </c>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="8">
+        <v>10000</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="B6" s="6">
-        <v>10000</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="D6" s="4">
         <v>0</v>
@@ -1962,15 +1957,15 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="9">
+        <v>5000</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="7">
-        <v>5000</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="7">
+      <c r="D7" s="9">
         <v>800</v>
       </c>
       <c r="E7" s="5"/>

</xml_diff>

<commit_message>
The never-silent principle held on the backend and died
</commit_message>
<xml_diff>
--- a/public/phare_template.xlsx
+++ b/public/phare_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\source\repos\phare\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF1FD77-5F8F-4B79-B909-CC029D5FB1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53BB672-F5BD-4178-B74D-D82385DE245C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Household" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="128">
   <si>
     <t>MONTHLY INCOME / REVENU MENSUEL</t>
   </si>
@@ -70,18 +70,12 @@
     <t>bi-weekly</t>
   </si>
   <si>
-    <t>Lineu</t>
-  </si>
-  <si>
     <t>One paycheque; paid every 2 weeks (26/yr)</t>
   </si>
   <si>
     <t>semi-monthly</t>
   </si>
   <si>
-    <t>Julia</t>
-  </si>
-  <si>
     <t>One paycheque; paid 15th &amp; 30th (24/yr)</t>
   </si>
   <si>
@@ -112,9 +106,6 @@
     <t>Family name / Nom de famille</t>
   </si>
   <si>
-    <t>Alff Graeff</t>
-  </si>
-  <si>
     <t>Province</t>
   </si>
   <si>
@@ -184,9 +175,6 @@
     <t>Ontario</t>
   </si>
   <si>
-    <t>Quebec + Ontario = tax gap, Lineu</t>
-  </si>
-  <si>
     <t>FIXED MONTHLY EXPENSES / DÉPENSES FIXES MENSUELLES</t>
   </si>
   <si>
@@ -403,9 +391,6 @@
     <t>September 2026</t>
   </si>
   <si>
-    <t>Brazil trip / Voyage Brésil</t>
-  </si>
-  <si>
     <t>Emergency fund / Fonds d'urgence</t>
   </si>
   <si>
@@ -422,6 +407,21 @@
   </si>
   <si>
     <t>Theme Park  trip / Visite d'un parc d'attractions</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Quebec + Ontario = tax gap, John</t>
+  </si>
+  <si>
+    <t>Europe trip / Voyage Europe</t>
   </si>
 </sst>
 </file>
@@ -441,63 +441,69 @@
       <sz val="14"/>
       <color rgb="FF0F2044"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF374151"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF6B7280"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0F2044"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF0F2044"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -864,7 +870,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -872,13 +878,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>7</v>
@@ -886,87 +892,87 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3">
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>13</v>
+        <v>124</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="D11" s="3"/>
     </row>
@@ -978,41 +984,41 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D15" s="3"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2">
@@ -1022,26 +1028,26 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>48</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>13</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1124,7 +1130,7 @@
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1135,41 +1141,41 @@
         <v>0</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" s="17">
         <v>0</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="17">
         <v>0</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1180,290 +1186,342 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
       <c r="E1" s="19"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="19"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C5" s="5">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="5">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="C9" s="5">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="B11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="5">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="C13" s="5">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="B14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="4">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="5">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="C16" s="4">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="5">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="E15" s="3"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="4">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="C17" s="5">
         <v>0</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
-      <c r="D22" s="8"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
-      <c r="D23" s="9"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1484,7 +1542,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1493,7 +1551,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1502,13 +1560,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>6</v>
@@ -1519,7 +1577,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B5" s="5">
         <v>800</v>
@@ -1528,13 +1586,13 @@
         <v>0</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B6" s="4">
         <v>350</v>
@@ -1543,13 +1601,13 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B7" s="5">
         <v>50</v>
@@ -1558,13 +1616,13 @@
         <v>0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B8" s="4">
         <v>150</v>
@@ -1573,13 +1631,13 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B9" s="5">
         <v>335</v>
@@ -1588,13 +1646,13 @@
         <v>0</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B10" s="4">
         <v>100</v>
@@ -1603,13 +1661,13 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B11" s="5">
         <v>100</v>
@@ -1618,13 +1676,13 @@
         <v>0</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B12" s="4">
         <v>100</v>
@@ -1633,13 +1691,13 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B13" s="5">
         <v>150</v>
@@ -1648,13 +1706,13 @@
         <v>0</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B14" s="4">
         <v>100</v>
@@ -1663,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E14" s="2"/>
     </row>
@@ -1706,7 +1764,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1716,7 +1774,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1726,7 +1784,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
@@ -1736,19 +1794,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>7</v>
@@ -1756,7 +1814,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B6" s="4">
         <v>3106.18</v>
@@ -1766,18 +1824,18 @@
         <v>258.8483333333333</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B7" s="5">
         <v>350</v>
@@ -1787,16 +1845,16 @@
         <v>29.166666666666668</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B8" s="4">
         <v>2000</v>
@@ -1806,18 +1864,18 @@
         <v>166.66666666666666</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B9" s="5">
         <v>200</v>
@@ -1827,18 +1885,18 @@
         <v>16.666666666666668</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B10" s="4">
         <v>300</v>
@@ -1848,16 +1906,16 @@
         <v>25</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B11" s="5">
         <v>600</v>
@@ -1867,18 +1925,18 @@
         <v>50</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B12" s="4">
         <v>1000</v>
@@ -1888,10 +1946,10 @@
         <v>83.333333333333329</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -1913,7 +1971,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B15" s="7">
         <f>SUM(B6:B14)</f>
@@ -1946,7 +2004,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1955,30 +2013,30 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B4" s="4">
         <v>5000</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D4" s="2">
         <v>0</v>
@@ -1987,7 +2045,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B5" s="5">
         <v>8000</v>
@@ -2002,7 +2060,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B6" s="4">
         <v>5000</v>
@@ -2017,7 +2075,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B7" s="5">
         <v>5000</v>

</xml_diff>

<commit_message>
Closes finding C1: unbounded prompt input on the two unauthenticated Anthropic-spending routes
</commit_message>
<xml_diff>
--- a/public/phare_template.xlsx
+++ b/public/phare_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\source\repos\phare\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lineu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542284D9-9C9C-4FAF-AFB1-1F372EDFDA39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Household" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Handoff — Household-sheet defects 1 & 2
</commit_message>
<xml_diff>
--- a/public/phare_template.xlsx
+++ b/public/phare_template.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="132">
   <si>
     <t>MONTHLY INCOME / REVENU MENSUEL</t>
   </si>
@@ -419,6 +419,21 @@
   </si>
   <si>
     <t>Europe trip / Voyage Europe</t>
+  </si>
+  <si>
+    <t>Employer province — Member 1 / Province de l'employeur — Membre 1</t>
+  </si>
+  <si>
+    <t>Employer province — Member 2 / Province de l'employeur — Membre 2</t>
+  </si>
+  <si>
+    <t>Jane — same province as residence / Jane — même province que la résidence</t>
+  </si>
+  <si>
+    <t>John — Quebec resident + Ontario employer = tax gap / John — résident du Québec + employeur ontarien = écart d'impôt</t>
+  </si>
+  <si>
+    <t>Member 2</t>
   </si>
 </sst>
 </file>
@@ -1025,26 +1040,26 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>43</v>
+        <v>128</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1688,7 +1703,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E12" s="2"/>
     </row>

</xml_diff>